<commit_message>
Ajustes carga masiva de reclamos
</commit_message>
<xml_diff>
--- a/importaciones/carga masiva desgravamen.xlsx
+++ b/importaciones/carga masiva desgravamen.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyectos\Global\importaciones\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7CCC0AF-AC83-473A-AF91-D1303B97B90C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C2B377C-88BF-4216-85B4-37AD664306C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="204" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="81">
   <si>
     <t>Ajustador</t>
   </si>
@@ -142,9 +142,6 @@
     <t>cob_116</t>
   </si>
   <si>
-    <t>12</t>
-  </si>
-  <si>
     <t>CL-EVR-CV1</t>
   </si>
   <si>
@@ -166,18 +163,6 @@
     <t>obs</t>
   </si>
   <si>
-    <t>4031</t>
-  </si>
-  <si>
-    <t>CV-000011</t>
-  </si>
-  <si>
-    <t>101</t>
-  </si>
-  <si>
-    <t>416468464</t>
-  </si>
-  <si>
     <t>VISA</t>
   </si>
   <si>
@@ -226,9 +211,6 @@
     <t>Prueba MSN-000052 dos coberturas</t>
   </si>
   <si>
-    <t>131513131</t>
-  </si>
-  <si>
     <t>3</t>
   </si>
   <si>
@@ -251,13 +233,43 @@
   </si>
   <si>
     <t>Prueba MSN-000052 duplicado</t>
+  </si>
+  <si>
+    <t>329</t>
+  </si>
+  <si>
+    <t>330</t>
+  </si>
+  <si>
+    <t>331</t>
+  </si>
+  <si>
+    <t>332</t>
+  </si>
+  <si>
+    <t>20-NT-20220-14596354</t>
+  </si>
+  <si>
+    <t>08-0657-00032</t>
+  </si>
+  <si>
+    <t>08-5555-44444</t>
+  </si>
+  <si>
+    <t>08-7777-88888</t>
+  </si>
+  <si>
+    <t>CV-000049</t>
+  </si>
+  <si>
+    <t>106</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <name val="Microsoft YaHei"/>
@@ -267,6 +279,12 @@
       <sz val="12"/>
       <color rgb="FF333333"/>
       <name val="Microsoft YaHei"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Microsoft YaHei"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -310,7 +328,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -319,6 +337,7 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -662,7 +681,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="17.25" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.5546875" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
@@ -674,7 +693,7 @@
     <col min="11" max="11" width="8.21875" style="1" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="10.21875" style="1" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="11.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="20.88671875" style="1" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="14.21875" style="1" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="13.77734375" style="1" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="7.109375" style="1" bestFit="1" customWidth="1"/>
@@ -815,91 +834,91 @@
       </c>
     </row>
     <row r="2" spans="1:40" ht="28.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>40</v>
+      <c r="A2">
+        <v>126</v>
       </c>
       <c r="B2"/>
       <c r="C2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D2" t="s">
         <v>41</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>42</v>
-      </c>
-      <c r="E2" t="s">
-        <v>43</v>
       </c>
       <c r="F2"/>
       <c r="G2" t="s">
+        <v>43</v>
+      </c>
+      <c r="H2" t="s">
         <v>44</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>45</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>46</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2">
+        <v>3952</v>
+      </c>
+      <c r="L2" t="s">
+        <v>79</v>
+      </c>
+      <c r="M2" t="s">
+        <v>71</v>
+      </c>
+      <c r="N2" t="s">
+        <v>75</v>
+      </c>
+      <c r="O2" t="s">
+        <v>44</v>
+      </c>
+      <c r="P2" t="s">
         <v>47</v>
       </c>
-      <c r="K2" t="s">
+      <c r="Q2" t="s">
         <v>48</v>
       </c>
-      <c r="L2" t="s">
+      <c r="R2" t="s">
         <v>49</v>
       </c>
-      <c r="M2" t="s">
+      <c r="S2" t="s">
         <v>50</v>
       </c>
-      <c r="N2" t="s">
+      <c r="T2" t="s">
         <v>51</v>
       </c>
-      <c r="O2" t="s">
-        <v>45</v>
-      </c>
-      <c r="P2" t="s">
+      <c r="U2" t="s">
         <v>52</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="V2" t="s">
         <v>53</v>
       </c>
-      <c r="R2" t="s">
+      <c r="W2" t="s">
         <v>54</v>
       </c>
-      <c r="S2" t="s">
+      <c r="X2" t="s">
         <v>55</v>
       </c>
-      <c r="T2" t="s">
+      <c r="Y2" t="s">
+        <v>41</v>
+      </c>
+      <c r="Z2" t="s">
         <v>56</v>
       </c>
-      <c r="U2" t="s">
+      <c r="AA2" t="s">
         <v>57</v>
       </c>
-      <c r="V2" t="s">
-        <v>58</v>
-      </c>
-      <c r="W2" t="s">
-        <v>59</v>
-      </c>
-      <c r="X2" t="s">
-        <v>60</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>42</v>
-      </c>
-      <c r="Z2" t="s">
-        <v>61</v>
-      </c>
-      <c r="AA2" t="s">
-        <v>62</v>
-      </c>
-      <c r="AB2"/>
+      <c r="AB2" s="4"/>
       <c r="AC2"/>
-      <c r="AD2"/>
+      <c r="AD2" s="4" t="s">
+        <v>80</v>
+      </c>
       <c r="AE2"/>
       <c r="AF2"/>
-      <c r="AG2">
-        <v>109</v>
-      </c>
+      <c r="AG2"/>
       <c r="AH2"/>
       <c r="AI2"/>
       <c r="AJ2"/>
@@ -909,85 +928,87 @@
       <c r="AN2"/>
     </row>
     <row r="3" spans="1:40" ht="28.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>40</v>
+      <c r="A3">
+        <v>126</v>
       </c>
       <c r="B3">
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="D3" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="E3" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="F3"/>
       <c r="G3" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="H3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="I3" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="J3"/>
-      <c r="K3" t="s">
-        <v>48</v>
+      <c r="K3">
+        <v>3952</v>
       </c>
       <c r="L3" t="s">
-        <v>49</v>
+        <v>79</v>
       </c>
       <c r="M3" t="s">
-        <v>68</v>
-      </c>
-      <c r="N3"/>
+        <v>72</v>
+      </c>
+      <c r="N3" t="s">
+        <v>76</v>
+      </c>
       <c r="O3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="P3" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="Q3" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="R3"/>
       <c r="S3" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="T3" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="U3" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="V3" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="W3" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="X3"/>
       <c r="Y3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="Z3" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="AA3" t="s">
-        <v>75</v>
-      </c>
-      <c r="AB3"/>
+        <v>69</v>
+      </c>
+      <c r="AB3" s="4"/>
       <c r="AC3"/>
-      <c r="AD3"/>
+      <c r="AD3" s="4" t="s">
+        <v>80</v>
+      </c>
       <c r="AE3"/>
       <c r="AF3"/>
-      <c r="AG3">
-        <v>109</v>
-      </c>
+      <c r="AG3"/>
       <c r="AH3"/>
       <c r="AI3"/>
       <c r="AJ3"/>
@@ -997,91 +1018,91 @@
       <c r="AN3"/>
     </row>
     <row r="4" spans="1:40" ht="28.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>40</v>
+      <c r="A4">
+        <v>126</v>
       </c>
       <c r="B4"/>
       <c r="C4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D4" t="s">
         <v>41</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>42</v>
-      </c>
-      <c r="E4" t="s">
-        <v>43</v>
       </c>
       <c r="F4"/>
       <c r="G4" t="s">
+        <v>43</v>
+      </c>
+      <c r="H4" t="s">
         <v>44</v>
       </c>
-      <c r="H4" t="s">
-        <v>45</v>
-      </c>
       <c r="I4" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="J4" t="s">
+        <v>46</v>
+      </c>
+      <c r="K4">
+        <v>3952</v>
+      </c>
+      <c r="L4" t="s">
+        <v>79</v>
+      </c>
+      <c r="M4" t="s">
+        <v>73</v>
+      </c>
+      <c r="N4" t="s">
+        <v>77</v>
+      </c>
+      <c r="O4" t="s">
+        <v>44</v>
+      </c>
+      <c r="P4" t="s">
         <v>47</v>
       </c>
-      <c r="K4" t="s">
+      <c r="Q4" t="s">
         <v>48</v>
       </c>
-      <c r="L4" t="s">
+      <c r="R4" t="s">
         <v>49</v>
       </c>
-      <c r="M4" t="s">
+      <c r="S4" t="s">
         <v>50</v>
       </c>
-      <c r="N4" t="s">
+      <c r="T4" t="s">
         <v>51</v>
       </c>
-      <c r="O4" t="s">
-        <v>45</v>
-      </c>
-      <c r="P4" t="s">
+      <c r="U4" t="s">
         <v>52</v>
       </c>
-      <c r="Q4" t="s">
+      <c r="V4" t="s">
         <v>53</v>
       </c>
-      <c r="R4" t="s">
+      <c r="W4" t="s">
         <v>54</v>
       </c>
-      <c r="S4" t="s">
+      <c r="X4" t="s">
         <v>55</v>
       </c>
-      <c r="T4" t="s">
+      <c r="Y4" t="s">
+        <v>41</v>
+      </c>
+      <c r="Z4" t="s">
         <v>56</v>
       </c>
-      <c r="U4" t="s">
+      <c r="AA4" t="s">
         <v>57</v>
       </c>
-      <c r="V4" t="s">
-        <v>58</v>
-      </c>
-      <c r="W4" t="s">
-        <v>59</v>
-      </c>
-      <c r="X4" t="s">
-        <v>60</v>
-      </c>
-      <c r="Y4" t="s">
-        <v>42</v>
-      </c>
-      <c r="Z4" t="s">
-        <v>61</v>
-      </c>
-      <c r="AA4" t="s">
-        <v>62</v>
-      </c>
-      <c r="AB4"/>
+      <c r="AB4" s="4"/>
       <c r="AC4"/>
-      <c r="AD4"/>
+      <c r="AD4" s="4" t="s">
+        <v>80</v>
+      </c>
       <c r="AE4"/>
       <c r="AF4"/>
-      <c r="AG4">
-        <v>109</v>
-      </c>
+      <c r="AG4"/>
       <c r="AH4"/>
       <c r="AI4"/>
       <c r="AJ4"/>
@@ -1091,91 +1112,91 @@
       <c r="AN4"/>
     </row>
     <row r="5" spans="1:40" ht="28.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>40</v>
+      <c r="A5">
+        <v>126</v>
       </c>
       <c r="B5"/>
       <c r="C5" t="s">
+        <v>40</v>
+      </c>
+      <c r="D5" t="s">
         <v>41</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>42</v>
-      </c>
-      <c r="E5" t="s">
-        <v>43</v>
       </c>
       <c r="F5"/>
       <c r="G5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="H5" s="3">
         <v>46294</v>
       </c>
       <c r="I5" t="s">
+        <v>45</v>
+      </c>
+      <c r="J5" t="s">
         <v>46</v>
       </c>
-      <c r="J5" t="s">
+      <c r="K5">
+        <v>3952</v>
+      </c>
+      <c r="L5" t="s">
+        <v>79</v>
+      </c>
+      <c r="M5" t="s">
+        <v>74</v>
+      </c>
+      <c r="N5" t="s">
+        <v>78</v>
+      </c>
+      <c r="O5" t="s">
+        <v>44</v>
+      </c>
+      <c r="P5" t="s">
         <v>47</v>
       </c>
-      <c r="K5" t="s">
+      <c r="Q5" t="s">
         <v>48</v>
       </c>
-      <c r="L5" t="s">
+      <c r="R5" t="s">
         <v>49</v>
       </c>
-      <c r="M5" t="s">
+      <c r="S5" t="s">
         <v>50</v>
       </c>
-      <c r="N5" t="s">
+      <c r="T5" t="s">
         <v>51</v>
       </c>
-      <c r="O5" t="s">
-        <v>45</v>
-      </c>
-      <c r="P5" t="s">
+      <c r="U5" t="s">
         <v>52</v>
       </c>
-      <c r="Q5" t="s">
+      <c r="V5" t="s">
         <v>53</v>
-      </c>
-      <c r="R5" t="s">
-        <v>54</v>
-      </c>
-      <c r="S5" t="s">
-        <v>55</v>
-      </c>
-      <c r="T5" t="s">
-        <v>56</v>
-      </c>
-      <c r="U5" t="s">
-        <v>57</v>
-      </c>
-      <c r="V5" t="s">
-        <v>58</v>
       </c>
       <c r="W5">
         <v>55</v>
       </c>
       <c r="X5" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="Y5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="Z5" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="AA5" t="s">
-        <v>62</v>
-      </c>
-      <c r="AB5"/>
+        <v>57</v>
+      </c>
+      <c r="AB5" s="4"/>
       <c r="AC5"/>
-      <c r="AD5"/>
+      <c r="AD5" s="4" t="s">
+        <v>80</v>
+      </c>
       <c r="AE5"/>
       <c r="AF5"/>
-      <c r="AG5">
-        <v>109</v>
-      </c>
+      <c r="AG5"/>
       <c r="AH5"/>
       <c r="AI5"/>
       <c r="AJ5"/>

</xml_diff>

<commit_message>
Ajustes de carga masiva y cierres de caja
</commit_message>
<xml_diff>
--- a/importaciones/carga masiva desgravamen.xlsx
+++ b/importaciones/carga masiva desgravamen.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyectos\Global\importaciones\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2FDA310-1139-4D18-84AF-61A7551A5A1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBFC8077-89C2-4466-A1DF-67DFA019EC6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="204" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="82">
   <si>
     <t>Ajustador</t>
   </si>
@@ -193,9 +193,6 @@
     <t>PR-1</t>
   </si>
   <si>
-    <t>Generales</t>
-  </si>
-  <si>
     <t>28/09/2026 14:30</t>
   </si>
   <si>
@@ -235,21 +232,12 @@
     <t>CV-000049</t>
   </si>
   <si>
-    <t>106</t>
-  </si>
-  <si>
-    <t>CL-EVR-CV12</t>
-  </si>
-  <si>
     <t>309</t>
   </si>
   <si>
     <t>310</t>
   </si>
   <si>
-    <t>311</t>
-  </si>
-  <si>
     <t>313</t>
   </si>
   <si>
@@ -259,10 +247,25 @@
     <t>08-7755-77170</t>
   </si>
   <si>
-    <t>4189131-2026131</t>
-  </si>
-  <si>
     <t>08-0345-00678</t>
+  </si>
+  <si>
+    <t>CL-EV-CV12</t>
+  </si>
+  <si>
+    <t>MUERTE NATURAL</t>
+  </si>
+  <si>
+    <t>CL-EV-CV13</t>
+  </si>
+  <si>
+    <t>CL-EV-CV14</t>
+  </si>
+  <si>
+    <t>319</t>
+  </si>
+  <si>
+    <t>88-8888-88888</t>
   </si>
 </sst>
 </file>
@@ -344,8 +347,10 @@
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -690,7 +695,7 @@
   <cols>
     <col min="1" max="1" width="18.21875" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.109375" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.5546875" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="7.33203125" style="1" bestFit="1" customWidth="1"/>
@@ -846,8 +851,8 @@
         <v>126</v>
       </c>
       <c r="B2"/>
-      <c r="C2" t="s">
-        <v>57</v>
+      <c r="C2" s="6" t="s">
+        <v>78</v>
       </c>
       <c r="D2" t="s">
         <v>40</v>
@@ -872,13 +877,13 @@
         <v>3952</v>
       </c>
       <c r="L2" t="s">
+        <v>69</v>
+      </c>
+      <c r="M2" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="M2" s="6" t="s">
+      <c r="N2" s="5" t="s">
         <v>73</v>
-      </c>
-      <c r="N2" s="6" t="s">
-        <v>77</v>
       </c>
       <c r="O2" t="s">
         <v>43</v>
@@ -921,11 +926,10 @@
       </c>
       <c r="AB2" s="4"/>
       <c r="AC2"/>
-      <c r="AD2" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="AE2"/>
-      <c r="AF2"/>
+      <c r="AD2" s="4"/>
+      <c r="AF2">
+        <v>108</v>
+      </c>
       <c r="AG2"/>
       <c r="AH2"/>
       <c r="AI2"/>
@@ -942,53 +946,53 @@
       <c r="B3">
         <v>1</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="D3" t="s">
         <v>57</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>58</v>
-      </c>
-      <c r="E3" t="s">
-        <v>59</v>
       </c>
       <c r="F3"/>
       <c r="G3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H3" t="s">
         <v>43</v>
       </c>
       <c r="I3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J3"/>
       <c r="K3">
         <v>3952</v>
       </c>
       <c r="L3" t="s">
-        <v>70</v>
-      </c>
-      <c r="M3" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="N3" s="5" t="s">
         <v>74</v>
-      </c>
-      <c r="N3" s="6" t="s">
-        <v>78</v>
       </c>
       <c r="O3" t="s">
         <v>43</v>
       </c>
       <c r="P3" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q3" t="s">
         <v>62</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>63</v>
       </c>
       <c r="R3"/>
       <c r="S3" t="s">
+        <v>63</v>
+      </c>
+      <c r="T3" t="s">
         <v>64</v>
-      </c>
-      <c r="T3" t="s">
-        <v>65</v>
       </c>
       <c r="U3" t="s">
         <v>51</v>
@@ -997,25 +1001,24 @@
         <v>52</v>
       </c>
       <c r="W3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="X3"/>
       <c r="Y3" t="s">
         <v>40</v>
       </c>
       <c r="Z3" t="s">
+        <v>66</v>
+      </c>
+      <c r="AA3" t="s">
         <v>67</v>
-      </c>
-      <c r="AA3" t="s">
-        <v>68</v>
       </c>
       <c r="AB3" s="4"/>
       <c r="AC3"/>
-      <c r="AD3" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="AE3"/>
-      <c r="AF3"/>
+      <c r="AD3" s="4"/>
+      <c r="AF3">
+        <v>108</v>
+      </c>
       <c r="AG3"/>
       <c r="AH3"/>
       <c r="AI3"/>
@@ -1031,7 +1034,7 @@
       </c>
       <c r="B4"/>
       <c r="C4" t="s">
-        <v>57</v>
+        <v>77</v>
       </c>
       <c r="D4" t="s">
         <v>40</v>
@@ -1047,7 +1050,7 @@
         <v>43</v>
       </c>
       <c r="I4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J4" t="s">
         <v>45</v>
@@ -1056,13 +1059,13 @@
         <v>3952</v>
       </c>
       <c r="L4" t="s">
-        <v>70</v>
-      </c>
-      <c r="M4" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="N4" s="6" t="s">
-        <v>79</v>
+        <v>69</v>
+      </c>
+      <c r="M4" t="s">
+        <v>80</v>
+      </c>
+      <c r="N4" t="s">
+        <v>81</v>
       </c>
       <c r="O4" t="s">
         <v>43</v>
@@ -1105,11 +1108,10 @@
       </c>
       <c r="AB4" s="4"/>
       <c r="AC4"/>
-      <c r="AD4" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="AE4"/>
-      <c r="AF4"/>
+      <c r="AD4" s="4"/>
+      <c r="AF4">
+        <v>108</v>
+      </c>
       <c r="AG4"/>
       <c r="AH4"/>
       <c r="AI4"/>
@@ -1124,8 +1126,8 @@
         <v>126</v>
       </c>
       <c r="B5"/>
-      <c r="C5" s="5" t="s">
-        <v>72</v>
+      <c r="C5" s="6" t="s">
+        <v>76</v>
       </c>
       <c r="D5" t="s">
         <v>40</v>
@@ -1150,13 +1152,13 @@
         <v>3952</v>
       </c>
       <c r="L5" t="s">
-        <v>70</v>
-      </c>
-      <c r="M5" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="N5" s="6" t="s">
-        <v>80</v>
+        <v>69</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="N5" s="5" t="s">
+        <v>75</v>
       </c>
       <c r="O5" t="s">
         <v>43</v>
@@ -1199,11 +1201,10 @@
       </c>
       <c r="AB5" s="4"/>
       <c r="AC5"/>
-      <c r="AD5" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="AE5"/>
-      <c r="AF5"/>
+      <c r="AD5" s="4"/>
+      <c r="AF5">
+        <v>108</v>
+      </c>
       <c r="AG5"/>
       <c r="AH5"/>
       <c r="AI5"/>

</xml_diff>

<commit_message>
Ajustes búsqueda de reclamos
</commit_message>
<xml_diff>
--- a/importaciones/carga masiva desgravamen.xlsx
+++ b/importaciones/carga masiva desgravamen.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyectos\Global\importaciones\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBFC8077-89C2-4466-A1DF-67DFA019EC6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CB430E6-0245-402B-8362-8E6D75124DA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="204" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -927,10 +927,10 @@
       <c r="AB2" s="4"/>
       <c r="AC2"/>
       <c r="AD2" s="4"/>
-      <c r="AF2">
-        <v>108</v>
-      </c>
-      <c r="AG2"/>
+      <c r="AF2"/>
+      <c r="AG2">
+        <v>109</v>
+      </c>
       <c r="AH2"/>
       <c r="AI2"/>
       <c r="AJ2"/>
@@ -1016,10 +1016,10 @@
       <c r="AB3" s="4"/>
       <c r="AC3"/>
       <c r="AD3" s="4"/>
-      <c r="AF3">
-        <v>108</v>
-      </c>
-      <c r="AG3"/>
+      <c r="AF3"/>
+      <c r="AG3">
+        <v>109</v>
+      </c>
       <c r="AH3"/>
       <c r="AI3"/>
       <c r="AJ3"/>
@@ -1109,10 +1109,10 @@
       <c r="AB4" s="4"/>
       <c r="AC4"/>
       <c r="AD4" s="4"/>
-      <c r="AF4">
-        <v>108</v>
-      </c>
-      <c r="AG4"/>
+      <c r="AF4"/>
+      <c r="AG4">
+        <v>109</v>
+      </c>
       <c r="AH4"/>
       <c r="AI4"/>
       <c r="AJ4"/>
@@ -1202,10 +1202,10 @@
       <c r="AB5" s="4"/>
       <c r="AC5"/>
       <c r="AD5" s="4"/>
-      <c r="AF5">
-        <v>108</v>
-      </c>
-      <c r="AG5"/>
+      <c r="AF5"/>
+      <c r="AG5">
+        <v>109</v>
+      </c>
       <c r="AH5"/>
       <c r="AI5"/>
       <c r="AJ5"/>

</xml_diff>